<commit_message>
Nav y Footer en color rojo
</commit_message>
<xml_diff>
--- a/Datos_Negocio.xlsx
+++ b/Datos_Negocio.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/26cb76602e667d66/Documents/proyectosMEGPaginaWeb/plantillaLeadMagnet/plantillaNueva/Plantilla_ProyectosMEG/Plantilla_PYMES/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ntact\Downloads\plantillaProyectosMEG-main\plantillaProyectosMEG-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="13_ncr:1_{963EA2D5-B6AB-433A-928E-C0326218B9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A27E0C9-2A68-40C5-A17A-F909461F55D2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59312877-011B-48ED-A272-0B297567BE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NAV" sheetId="11" r:id="rId1"/>
@@ -1516,10 +1516,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
   <a:themeElements>
@@ -1786,7 +1782,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>106</v>
+        <v>35</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>12</v>
@@ -4557,7 +4553,7 @@
         <v>125</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>126</v>

</xml_diff>